<commit_message>
Use game events instead of patches
</commit_message>
<xml_diff>
--- a/package/translations.xlsx
+++ b/package/translations.xlsx
@@ -471,17 +471,17 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Controls conversion behavior and saved joined-god progress. Joined-god progress is local-save oriented and may not travel with Steam Cloud.</t>
+          <t>Controls conversion behavior and saved joined-god progress. Joined-god progress is stored in the current save.</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>改宗と加入済み神の進行保存を設定します。保存データはローカル保存向けで、Steam Cloudには含まれない場合があります。</t>
+          <t>改宗と加入済み神の進行保存を設定します。加入済み神の進行は現在のセーブに保存されます。</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>控制改宗和已加入神明进度。该进度偏向本地存档，Steam Cloud 可能不会同步。</t>
+          <t>控制改宗和已加入神明进度。已加入神明进度会保存在当前存档中。</t>
         </is>
       </c>
     </row>
@@ -735,17 +735,17 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Previous gods stay joined when converting. Saved piety, days, and reward history are restored per local save.</t>
+          <t>Previous gods stay joined when converting. Saved piety, days, and reward history are restored per save.</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>改宗後も以前の神を加入済みにします。信仰心、日数、報酬履歴をローカル保存ごとに復元します。</t>
+          <t>改宗後も以前の神を加入済みにします。信仰心、日数、報酬履歴をセーブごとに復元します。</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>改宗后保留已加入神明。按本地存档恢复虔诚、天数和奖励历史。</t>
+          <t>改宗后保留已加入神明。按存档恢复虔诚、天数和奖励历史。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated for EA 23.307 Stable. Fixed saved piety being reduced when multi-god joining is off, and fixed joined Eyth bonuses not applying for Demigod players.
EA 23.307 Stable に対応しました。複数信仰がオフの時に保存済み信仰心が減る問題と、半神で加入済みエイスの恩恵が適用されない問題を修正しました。

已更新至 EA 23.307 Stable。修正了多神明加入关闭时保存虔诚被降低的问题，并修正半神玩家的已加入艾斯加成不生效的问题。
</commit_message>
<xml_diff>
--- a/package/translations.xlsx
+++ b/package/translations.xlsx
@@ -471,17 +471,17 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Controls conversion behavior and saved joined-god progress. Joined-god progress is stored in the current save.</t>
+          <t>Controls conversion behavior and saved joined-god progress. When off, saved non-current god progress is ignored for gameplay but kept in the save without being erased or reduced.</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>改宗と加入済み神の進行保存を設定します。加入済み神の進行は現在のセーブに保存されます。</t>
+          <t>改宗と加入済み神の進行保存を設定します。オフの間、現在信仰ではない神の保存済み進行はゲームプレイでは無視されますが、セーブ内では削除・減少されずに保持されます。</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>控制改宗和已加入神明进度。已加入神明进度会保存在当前存档中。</t>
+          <t>控制改宗和已加入神明进度。关闭时，非当前神明的保存进度会在玩法中被忽略，但仍保留在存档中，不会被删除或降低。</t>
         </is>
       </c>
     </row>
@@ -647,17 +647,17 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Controls joined-god bonuses, faith resistance caps, god artifact faction effects, duplicate god artifacts, Eyth cleanup, and apostle infighting.</t>
+          <t>Controls joined-god bonuses, faith resistance caps, god artifact faction effects, duplicate god artifacts, Eyth cleanup, and apostle infighting. Non-current god effects require Allow Joining Multiple Religions and saved joined state.</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>加入済み神の恩恵、信仰耐性上限、神アーティファクト陣営効果、重複、エイス整理、使徒争いを設定します。</t>
+          <t>加入済み神の恩恵、信仰耐性上限、神アーティファクト陣営効果、重複、エイス整理、使徒争いを設定します。現在信仰ではない神の効果には Allow Joining Multiple Religions と保存済み加入状態が必要です。</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>控制已加入神明加成、信仰抗性上限、神器阵营效果、重复神器、艾斯清理和使徒内斗。</t>
+          <t>控制已加入神明加成、信仰抗性上限、神器阵营效果、重复神器、艾斯清理和使徒内斗。非当前神明效果需要启用 Allow Joining Multiple Religions 并已有保存的加入状态。</t>
         </is>
       </c>
     </row>
@@ -691,17 +691,17 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Controls extra joined-god prayer revelations and their chance. Vanilla mode keeps only the current faith.</t>
+          <t>Controls extra joined-god prayer revelations and their chance. Vanilla mode keeps only the current faith. Non-current gods require Allow Joining Multiple Religions and saved joined state.</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>加入済み神による追加の祈りの啓示と発生率を設定します。Vanillaは現在信仰のみです。</t>
+          <t>加入済み神による追加の祈りの啓示と発生率を設定します。Vanillaは現在信仰のみです。現在信仰ではない神には Allow Joining Multiple Religions と保存済み加入状態が必要です。</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>控制已加入神明的额外祈祷启示及其几率。Vanilla 仅使用当前信仰。</t>
+          <t>控制已加入神明的额外祈祷启示及其几率。Vanilla 仅使用当前信仰。非当前神明需要启用 Allow Joining Multiple Religions 并已有保存的加入状态。</t>
         </is>
       </c>
     </row>
@@ -735,17 +735,17 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Previous gods stay joined when converting. Saved piety, days, and reward history are restored per save.</t>
+          <t>Previous gods stay joined when converting. Saved piety, days, and reward history are restored per save while enabled. When off, saved progress is ignored for gameplay, not erased or reduced.</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>改宗後も以前の神を加入済みにします。信仰心、日数、報酬履歴をセーブごとに復元します。</t>
+          <t>改宗後も以前の神を加入済みにします。有効時は信仰心、日数、報酬履歴をセーブごとに復元します。オフの間は保存済み進行をゲームプレイでは無視しますが、削除・減少しません。</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>改宗后保留已加入神明。按存档恢复虔诚、天数和奖励历史。</t>
+          <t>改宗后保留已加入神明。启用时按存档恢复虔诚、天数和奖励历史。关闭时会在玩法中忽略保存进度，但不会删除或降低。</t>
         </is>
       </c>
     </row>
@@ -867,17 +867,17 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Offerings at a joined god's own altar can increase that god's piety even when they are not current faith.</t>
+          <t>Offerings at a joined god's own altar can increase that god's piety even when they are not current faith. Requires Allow Joining Multiple Religions and saved joined state.</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>加入済み神自身の祭壇なら、現在信仰でなくてもその神の信仰心を増やします。</t>
+          <t>加入済み神自身の祭壇なら、現在信仰でなくてもその神の信仰心を増やします。Allow Joining Multiple Religions と保存済み加入状態が必要です。</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>在已加入神明自己的祭坛献祭时，即使不是当前信仰也增加该神明虔诚。</t>
+          <t>在已加入神明自己的祭坛献祭时，即使不是当前信仰也增加该神明虔诚。需要启用 Allow Joining Multiple Religions 并已有保存的加入状态。</t>
         </is>
       </c>
     </row>
@@ -1307,17 +1307,17 @@
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Prayer piety also applies to joined non-current gods.</t>
+          <t>Prayer piety also applies to joined non-current gods. Non-current gods require Allow Joining Multiple Religions and saved joined state.</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>祈りの信仰心を現在信仰でない加入済み神にも適用します。</t>
+          <t>祈りの信仰心を現在信仰でない加入済み神にも適用します。現在信仰ではない神には Allow Joining Multiple Religions と保存済み加入状態が必要です。</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>祈祷虔诚也应用到非当前的已加入神明。</t>
+          <t>祈祷虔诚也应用到非当前的已加入神明。非当前神明需要启用 Allow Joining Multiple Religions 并已有保存的加入状态。</t>
         </is>
       </c>
     </row>
@@ -1395,17 +1395,17 @@
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>Prayer checks reward eligibility for joined non-current gods too.</t>
+          <t>Prayer checks reward eligibility for joined non-current gods too. Non-current gods require Allow Joining Multiple Religions and saved joined state.</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>祈りで現在信仰でない加入済み神の報酬も確認します。</t>
+          <t>祈りで現在信仰でない加入済み神の報酬も確認します。現在信仰ではない神には Allow Joining Multiple Religions と保存済み加入状態が必要です。</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>祈祷也检查非当前已加入神明的奖励资格。</t>
+          <t>祈祷也检查非当前已加入神明的奖励资格。非当前神明需要启用 Allow Joining Multiple Religions 并已有保存的加入状态。</t>
         </is>
       </c>
     </row>
@@ -1615,17 +1615,17 @@
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>Adds faith bonus elements from joined non-current gods. This is a powerful stacking option.</t>
+          <t>Adds faith bonus elements from joined non-current gods. Requires Allow Joining Multiple Religions and saved joined state for those gods.</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>現在信仰でない加入済み神の恩恵も追加します。強力な重複オプションです。</t>
+          <t>現在信仰でない加入済み神の恩恵も追加します。その神に対する Allow Joining Multiple Religions と保存済み加入状態が必要です。</t>
         </is>
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>添加非当前已加入神明的信仰加成。这是强力叠加选项。</t>
+          <t>添加非当前已加入神明的信仰加成。需要启用 Allow Joining Multiple Religions，并且这些神明已有保存的加入状态。</t>
         </is>
       </c>
     </row>
@@ -1703,17 +1703,17 @@
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>Joined god artifacts can provide faction effects even when that god is not current faith.</t>
+          <t>Joined god artifacts can provide faction effects even when that god is not current faith. Non-current gods require Allow Joining Multiple Religions and saved joined state.</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>加入済み神の神アーティファクトは、現在信仰でなくても陣営効果を発揮できます。</t>
+          <t>加入済み神の神アーティファクトは、現在信仰でなくても陣営効果を発揮できます。現在信仰でない神には Allow Joining Multiple Religions と保存済み加入状態が必要です。</t>
         </is>
       </c>
       <c r="D61" s="8" t="inlineStr">
         <is>
-          <t>已加入神明的神器即使不是当前信仰也可提供阵营效果。</t>
+          <t>已加入神明的神器即使不是当前信仰也可提供阵营效果。非当前神明需要启用 Allow Joining Multiple Religions 并已有保存的加入状态。</t>
         </is>
       </c>
     </row>
@@ -1879,17 +1879,17 @@
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>Joined gods may answer prayer revelations according to Revelation Mode.</t>
+          <t>Joined gods may answer prayer revelations according to Revelation Mode. Non-current gods require Allow Joining Multiple Religions and saved joined state.</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>Revelation Modeに従って加入済み神が祈りの啓示に応じることがあります。</t>
+          <t>Revelation Modeに従って加入済み神が祈りの啓示に応じることがあります。現在信仰ではない神には Allow Joining Multiple Religions と保存済み加入状態が必要です。</t>
         </is>
       </c>
       <c r="D69" s="8" t="inlineStr">
         <is>
-          <t>已加入神明可按启示模式回应祈祷启示。</t>
+          <t>已加入神明可按启示模式回应祈祷启示。非当前神明需要启用 Allow Joining Multiple Religions 并已有保存的加入状态。</t>
         </is>
       </c>
     </row>

</xml_diff>